<commit_message>
docs: update UAT plan + guide + deployment plan for the LIVE Trust hand-off
- UAT workbook Capacity & Trust: TRU-011 (engine now remote/live), TRU-012
  (hand-off happy path replaces 'no handoff today'), new TRU-033 (return +
  read-back) + TRU-034 (availability gate / kill switch); coverage summary reworded.
- UAT_Guide.md: 'things to know' now describes the live hand-off, not a dormant seam.
- PRODUCTION_DEPLOYMENT_PLAN.md: added the Kuja Trust hand-off env vars
  (KUJA_TRUST_HANDOFF_SECRET + KUJA_TRUST_SERVICE_TOKEN shared on BOTH services,
  KUJA_TRUST_BASE_URL/ENGINE/GRANT_BASE_URL on Grant) to the launch checklist.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/uat/Kuja_UAT_Test_Plan.xlsx
+++ b/docs/uat/Kuja_UAT_Test_Plan.xlsx
@@ -20,7 +20,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'NGO Journey'!$A$2:$O$54</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Capacity &amp; Trust'!$A$2:$O$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Capacity &amp; Trust'!$A$2:$O$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Donor Journey'!$A$2:$O$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Reviewer Journey'!$A$2:$O$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Admin &amp; Platform'!$A$2:$O$22</definedName>
@@ -2772,12 +2772,12 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>34</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>16</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -2972,12 +2972,12 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>195</t>
+          <t>197</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>92</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
@@ -3043,7 +3043,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Capacity &amp; Trust: in-app assessment + Passport publish/share/verify; the standalone Kuja Trust app (7 C4C domains, evidence room, screening, self-declared vs verified-clear, languages/RTL, low-data mode); and the (currently dormant) Grant↔Trust service seam.</t>
+          <t>Capacity &amp; Trust: in-app assessment + Passport publish/share/verify; the standalone Kuja Trust app (7 C4C domains, evidence room, screening, self-declared vs verified-clear, languages/RTL, low-data mode); and the LIVE Grant↔Trust hand-off + service read-back.</t>
         </is>
       </c>
     </row>
@@ -6242,7 +6242,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O34"/>
+  <dimension ref="A1:O36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6933,7 +6933,7 @@
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>Seam diagnostics show engine mode</t>
+          <t>Seam diagnostics show the engine is LIVE</t>
         </is>
       </c>
       <c r="D13" s="22" t="inlineStr">
@@ -6968,7 +6968,7 @@
       </c>
       <c r="J13" s="12" t="inlineStr">
         <is>
-          <t>Reports engine mode (default 'local'), and whether remote Trust is configured/reachable — expected DORMANT unless KUJA_TRUST_* env vars are set.</t>
+          <t>For the Kuja tenant with the hand-off configured: mode='remote', remote_configured=true, remote_reachable=true. (If the shared secret / engine are unset it falls back to 'local' — the kill switch.)</t>
         </is>
       </c>
       <c r="K13" s="12" t="inlineStr"/>
@@ -6990,17 +6990,17 @@
       </c>
       <c r="C14" s="16" t="inlineStr">
         <is>
-          <t>No user-facing Grant→Trust handoff today</t>
-        </is>
-      </c>
-      <c r="D14" s="21" t="inlineStr">
-        <is>
-          <t>Edge</t>
+          <t>Hand-off: Grant → Kuja Trust assessment (no 2nd login)</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>Happy</t>
         </is>
       </c>
       <c r="E14" s="18" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="F14" s="16" t="inlineStr">
@@ -7010,7 +7010,7 @@
       </c>
       <c r="G14" s="16" t="inlineStr">
         <is>
-          <t>Signed in</t>
+          <t>Signed in as NGO on /trust; hand-off configured</t>
         </is>
       </c>
       <c r="H14" s="16" t="inlineStr">
@@ -7020,12 +7020,13 @@
       </c>
       <c r="I14" s="16" t="inlineStr">
         <is>
-          <t>1. Look across the Grant UI for any link/redirect/SSO to kuja-app-production (Trust app)</t>
+          <t>1. On /trust click 'Complete your capacity assessment in Kuja Trust'
+2. Follow the redirect</t>
         </is>
       </c>
       <c r="J14" s="16" t="inlineStr">
         <is>
-          <t>There is NO in-UI handoff currently; the 'real' capacity assessment is completed directly in the standalone Trust app. (Document this as expected pilot behaviour.)</t>
+          <t>You land on the Assessment tab in Kuja Trust with NO second login (a short-lived signed link binds your org); a 'Return to your application' bar is shown. Your Trust org is created/linked on first arrival (external_ref=grant:&lt;id&gt;).</t>
         </is>
       </c>
       <c r="K14" s="16" t="inlineStr"/>
@@ -8179,13 +8180,129 @@
       <c r="N34" s="16" t="inlineStr"/>
       <c r="O34" s="16" t="inlineStr"/>
     </row>
+    <row r="35">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
+          <t>TRU-033</t>
+        </is>
+      </c>
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>Grant↔Trust</t>
+        </is>
+      </c>
+      <c r="C35" s="12" t="inlineStr">
+        <is>
+          <t>Return to grant + result reads back</t>
+        </is>
+      </c>
+      <c r="D35" s="13" t="inlineStr">
+        <is>
+          <t>Happy</t>
+        </is>
+      </c>
+      <c r="E35" s="14" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F35" s="12" t="inlineStr">
+        <is>
+          <t>NGO · fatima@amani.org</t>
+        </is>
+      </c>
+      <c r="G35" s="12" t="inlineStr">
+        <is>
+          <t>Completed a hand-off assessment in Kuja Trust (TRU-012)</t>
+        </is>
+      </c>
+      <c r="H35" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I35" s="12" t="inlineStr">
+        <is>
+          <t>1. In Kuja Trust click 'Return to your application'
+2. Land back on Grant /trust (?from=trust)</t>
+        </is>
+      </c>
+      <c r="J35" s="12" t="inlineStr">
+        <is>
+          <t>You return to the Grant app; a 'Welcome back from Kuja Trust' banner shows and the capacity &amp; due-diligence status now reflects the Trust assessment (the profile is served with source='trust').</t>
+        </is>
+      </c>
+      <c r="K35" s="12" t="inlineStr"/>
+      <c r="L35" s="14" t="inlineStr"/>
+      <c r="M35" s="12" t="inlineStr"/>
+      <c r="N35" s="12" t="inlineStr"/>
+      <c r="O35" s="12" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="15" t="inlineStr">
+        <is>
+          <t>TRU-034</t>
+        </is>
+      </c>
+      <c r="B36" s="16" t="inlineStr">
+        <is>
+          <t>Grant↔Trust</t>
+        </is>
+      </c>
+      <c r="C36" s="16" t="inlineStr">
+        <is>
+          <t>Hand-off availability gate / kill switch</t>
+        </is>
+      </c>
+      <c r="D36" s="21" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="E36" s="18" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F36" s="16" t="inlineStr">
+        <is>
+          <t>NGO · fatima@amani.org</t>
+        </is>
+      </c>
+      <c r="G36" s="16" t="inlineStr">
+        <is>
+          <t>Signed in as NGO</t>
+        </is>
+      </c>
+      <c r="H36" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I36" s="16" t="inlineStr">
+        <is>
+          <t>1. Call GET /api/trust/handoff/available
+2. (Ops) confirm the CTA hides if KUJA_TRUST_HANDOFF_SECRET is unset</t>
+        </is>
+      </c>
+      <c r="J36" s="16" t="inlineStr">
+        <is>
+          <t>Returns available:true only when the hand-off is configured for the Kuja tenant; with the secret unset the CTA is hidden, /handoff is inert, and the app falls back to its own in-app assessment — non-destructive kill switch.</t>
+        </is>
+      </c>
+      <c r="K36" s="16" t="inlineStr"/>
+      <c r="L36" s="18" t="inlineStr"/>
+      <c r="M36" s="16" t="inlineStr"/>
+      <c r="N36" s="16" t="inlineStr"/>
+      <c r="O36" s="16" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:O34"/>
+  <autoFilter ref="A2:O36"/>
   <mergeCells count="1">
     <mergeCell ref="A1:O1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="L3:L34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L3:L36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not run,In progress"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>